<commit_message>
feat(inquiry): rename category select to '진료과 선택' + add '기타' option
- InquiryModal select label: Select category → Select department (진료과 선택, all langs)
- add '기타'/'Other' to modal category options
- regenerate i18n Excel

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/i18n/strings.xlsx
+++ b/docs/i18n/strings.xlsx
@@ -36907,22 +36907,22 @@
       </c>
       <c r="B8" s="3" t="inlineStr">
         <is>
-          <t>Select category</t>
+          <t>Select department</t>
         </is>
       </c>
       <c r="C8" s="3" t="inlineStr">
         <is>
-          <t>병원 구분 선택</t>
+          <t>진료과 선택</t>
         </is>
       </c>
       <c r="D8" s="4" t="inlineStr">
         <is>
-          <t>اختر الفئة</t>
+          <t>اختر التخصص</t>
         </is>
       </c>
       <c r="E8" s="3" t="inlineStr">
         <is>
-          <t>病院区分を選択</t>
+          <t>診療科を選択</t>
         </is>
       </c>
       <c r="F8" s="2" t="inlineStr">

</xml_diff>

<commit_message>
feat(contact): align /contact category select to modal — 진료과 label + 기타 option
- i18n 'Hospital category' → Department/진료과 (all langs)
- add 기타/Other to /contact category options
- regenerate i18n Excel

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/i18n/strings.xlsx
+++ b/docs/i18n/strings.xlsx
@@ -39403,22 +39403,22 @@
       </c>
       <c r="B86" s="3" t="inlineStr">
         <is>
-          <t>Hospital category</t>
+          <t>Department</t>
         </is>
       </c>
       <c r="C86" s="3" t="inlineStr">
         <is>
-          <t>병원 구분</t>
+          <t>진료과</t>
         </is>
       </c>
       <c r="D86" s="4" t="inlineStr">
         <is>
-          <t>تصنيف المستشفى</t>
+          <t>التخصص</t>
         </is>
       </c>
       <c r="E86" s="3" t="inlineStr">
         <is>
-          <t>病院区分</t>
+          <t>診療科</t>
         </is>
       </c>
       <c r="F86" s="2" t="inlineStr">

</xml_diff>